<commit_message>
Lambda WMS 2023-10-24 迭代1.16 质检单 开发
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/b2bsoExport.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/b2bsoExport.xlsx
@@ -54,14 +54,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>结算币别</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否含税</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>备注</t>
   </si>
   <si>
@@ -262,6 +254,239 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
+      <t>地址类型</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>收款条件</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SKU</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>销售数量</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>销售单价</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>是否赠品</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>是否补发</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>单据日期</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>单据类型</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>序号</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>交货方式</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -287,7 +512,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>地址类型</t>
+      <t>结算币别</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -312,190 +537,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>收款条件</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SKU</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>销售数量</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>销售单价</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>是否赠品</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>是否补发</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>备注</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>单据日期</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>单据类型</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>序号</t>
+      <t>是否含税</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -946,28 +988,28 @@
   <sheetData>
     <row r="1" spans="1:36" s="1" customFormat="1" ht="20.25" customHeight="1" thickBot="1">
       <c r="A1" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>1</v>
@@ -976,10 +1018,10 @@
         <v>2</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>3</v>
@@ -994,13 +1036,13 @@
         <v>6</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="T1" s="3" t="s">
         <v>8</v>
@@ -1009,49 +1051,49 @@
         <v>9</v>
       </c>
       <c r="V1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="AB1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AC1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="AD1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:36">
@@ -1059,6 +1101,11 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y1:Y1048576">
+      <formula1>"是,否"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Lambda  2023-10-24 迭代1.16 开发
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/b2bsoExport.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/b2bsoExport.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$AG$1:$AG$2</definedName>
+  </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
@@ -60,10 +63,6 @@
     <t>税率(%)</t>
   </si>
   <si>
-    <t>是否关闭</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <t>*</t>
     </r>
@@ -538,6 +537,31 @@
         <scheme val="minor"/>
       </rPr>
       <t>是否含税</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>是否关闭</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -988,28 +1012,28 @@
   <sheetData>
     <row r="1" spans="1:36" s="1" customFormat="1" ht="20.25" customHeight="1" thickBot="1">
       <c r="A1" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>15</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>1</v>
@@ -1018,10 +1042,10 @@
         <v>2</v>
       </c>
       <c r="K1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>3</v>
@@ -1036,13 +1060,13 @@
         <v>6</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T1" s="3" t="s">
         <v>8</v>
@@ -1051,46 +1075,46 @@
         <v>9</v>
       </c>
       <c r="V1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AB1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AB1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="AF1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="AG1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AH1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AH1" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="AI1" s="3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="AJ1" s="3" t="s">
         <v>10</v>
@@ -1101,9 +1125,24 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y1:Y1048576">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y1:Y1048576 G1:G1048576 AG1:AG1048576 AH1:AH1048576 AI1:AI1048576">
       <formula1>"是,否"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576">
+      <formula1>"B2B订单,售后订单-补/换/赠"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O1048576">
+      <formula1>"EXW,FOB,FCA,DAP,DDU,DDP"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W1:W1048576">
+      <formula1>"自提,发货"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z1:Z1048576">
+      <formula1>"货代地址,收货地址,公司地址"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA1:AA1048576">
+      <formula1>"网店销售收款,预收100%,货到收款,多到期日(按金额),月结30天,分期付款,30天后收款"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>